<commit_message>
data: hourly update 2026-07-11 16:04Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-11.xlsx
+++ b/data/output/workbook/2026-07-11.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28</t>
+          <t>2026-07-11 12:03</t>
         </is>
       </c>
     </row>
@@ -8918,7 +8918,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6507000000000001</v>
+        <v>0.6501</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-186</v>
@@ -8948,7 +8948,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -186). Your call.</t>
+          <t>Model 65.0% (fair -186). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8965,12 +8965,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8980,17 +8980,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers +1.5</t>
+          <t>Athletics +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.6331</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-129</v>
+        <v>-173</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9014,7 +9014,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 63.3% (fair -173). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9041,22 +9041,22 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Boston Red Sox +1.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5531</v>
+        <v>0.6224000000000001</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-124</v>
+        <v>-165</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>126</v>
+        <v>162</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9080,7 +9080,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9097,32 +9097,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Tampa Bay Rays</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Milwaukee Brewers +1.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5447</v>
+        <v>0.5589999999999999</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-120</v>
+        <v>-127</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9146,7 +9146,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 55.9% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9163,32 +9163,32 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates -1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.437</v>
+        <v>0.5705</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>129</v>
+        <v>-133</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>178</v>
+        <v>117</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9229,12 +9229,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Seattle Mariners @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -9244,17 +9244,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5564</v>
+        <v>0.5447</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-125</v>
+        <v>-120</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9305,22 +9305,22 @@
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5225</v>
+        <v>0.441</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-109</v>
+        <v>127</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>122</v>
+        <v>178</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 44.1% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9361,12 +9361,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -9376,17 +9376,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5033</v>
+        <v>0.5557000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-101</v>
+        <v>-125</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9410,7 +9410,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9427,12 +9427,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Atlanta Dream</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -9442,17 +9442,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5622</v>
+        <v>0.5317000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-128</v>
+        <v>-114</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>122</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9493,32 +9493,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Atlanta Dream</t>
+          <t>Boston Red Sox @ New York Mets</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire +13.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5383</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-126</v>
+        <v>-117</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-103</v>
+        <v>117</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9542,7 +9542,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9559,32 +9559,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Portland Fire @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Portland Fire +14.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6361</v>
+        <v>0.5656</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-175</v>
+        <v>-130</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-138</v>
+        <v>105</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 63.6% (fair -175). Your call.</t>
+          <t>Model 56.6% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9625,12 +9625,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -9644,13 +9644,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5347</v>
+        <v>0.4949</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-115</v>
+        <v>102</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>105</v>
+        <v>133</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -9674,7 +9674,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9686,34 +9686,34 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4901</v>
+        <v>0.5051</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>104</v>
+        <v>-102</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>122</v>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9757,12 +9757,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>New York Liberty @ Toronto Tempo</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9772,17 +9772,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6204000000000001</v>
+        <v>0.5699000000000001</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-163</v>
+        <v>-133</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-133</v>
+        <v>-108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9823,12 +9823,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Detroit Tigers</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>22:10</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9838,17 +9838,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4781</v>
+        <v>0.6361</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>109</v>
+        <v>-175</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>127</v>
+        <v>-138</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9872,7 +9872,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 63.6% (fair -175). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9884,37 +9884,37 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Las Vegas Aces</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury +10.5</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5356000000000001</v>
+        <v>0.4901</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-115</v>
+        <v>104</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9938,7 +9938,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9950,37 +9950,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5734</v>
+        <v>0.5295</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-134</v>
+        <v>-113</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-113</v>
+        <v>105</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 52.9% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10031,22 +10031,22 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5067</v>
+        <v>0.4776</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-103</v>
+        <v>109</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10070,7 +10070,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10087,32 +10087,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Las Vegas Aces</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Over 170</t>
+          <t>Miami Marlins -1.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.533</v>
+        <v>0.4218</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-114</v>
+        <v>137</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10136,7 +10136,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10153,32 +10153,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Washington Nationals +1.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4967</v>
+        <v>0.509</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>101</v>
+        <v>-104</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10202,7 +10202,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10214,37 +10214,37 @@
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>New York Liberty @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins -1.5</t>
+          <t>New York Liberty</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4255</v>
+        <v>0.6195999999999999</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>135</v>
+        <v>-163</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>150</v>
+        <v>-138</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10268,7 +10268,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 62.0% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10280,37 +10280,37 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever @ Las Vegas Aces</t>
+          <t>Philadelphia Phillies @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.3818</v>
+        <v>0.4885</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>178</v>
+        <v>116</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 38.2% (fair +162). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10346,37 +10346,37 @@
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>New York Liberty @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Under 173.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5923</v>
+        <v>0.5049</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-145</v>
+        <v>-102</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-127</v>
+        <v>108</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10400,7 +10400,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10417,7 +10417,7 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -10427,22 +10427,22 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals +1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5118</v>
+        <v>0.4705</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-105</v>
+        <v>113</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -10466,7 +10466,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 47.1% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -10643,10 +10643,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.3690861999999995</v>
+        <v>0.3587399999999999</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>113</v>
@@ -10673,7 +10673,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 36.9% (fair +171). Your call.</t>
+          <t>Model 35.9% (fair +179). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -10709,13 +10709,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6309138000000005</v>
+        <v>0.6412600000000001</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-171</v>
+        <v>-179</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -10739,7 +10739,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 63.1% (fair -171). Your call.</t>
+          <t>Model 64.1% (fair -179). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10775,10 +10775,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4775</v>
+        <v>0.4683</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>105</v>
@@ -10805,7 +10805,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10841,10 +10841,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5225</v>
+        <v>0.5317000000000001</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-109</v>
+        <v>-114</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>122</v>
@@ -10871,7 +10871,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10907,10 +10907,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.437</v>
+        <v>0.441</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>178</v>
@@ -10937,7 +10937,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 43.7% (fair +129). Your call.</t>
+          <t>Model 44.1% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10973,10 +10973,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5589999999999999</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-129</v>
+        <v>-127</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>178</v>
@@ -11003,7 +11003,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 56.3% (fair -129). Your call.</t>
+          <t>Model 55.9% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -11111,7 +11111,7 @@
         <v>-120</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -11171,10 +11171,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5347</v>
+        <v>0.5295</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-115</v>
+        <v>-113</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>105</v>
@@ -11201,7 +11201,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 52.9% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11237,10 +11237,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4653</v>
+        <v>0.4705</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>122</v>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 47.1% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11303,7 +11303,7 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.3493</v>
+        <v>0.3499</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>186</v>
@@ -11333,7 +11333,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 34.9% (fair +186). Your call.</t>
+          <t>Model 35.0% (fair +186). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -11369,7 +11369,7 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6507000000000001</v>
+        <v>0.6501</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>-186</v>
@@ -11399,7 +11399,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -186). Your call.</t>
+          <t>Model 65.0% (fair -186). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11441,7 +11441,7 @@
         <v>286</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -11567,13 +11567,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5033</v>
+        <v>0.4949</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-101</v>
+        <v>102</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -11633,13 +11633,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4967</v>
+        <v>0.5051</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>101</v>
+        <v>-102</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11699,13 +11699,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4648</v>
+        <v>0.4583</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11765,13 +11765,13 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5352</v>
+        <v>0.5417000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-115</v>
+        <v>-118</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-127</v>
+        <v>-125</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -11795,7 +11795,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11831,13 +11831,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4489288</v>
+        <v>0.452091</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -11861,7 +11861,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11897,13 +11897,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5510712</v>
+        <v>0.547909</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-123</v>
+        <v>-121</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11959,17 +11959,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4744</v>
+        <v>0.5705</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>111</v>
+        <v>-133</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12025,17 +12025,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4384000000000001</v>
+        <v>0.4295</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -12059,7 +12059,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 43.8% (fair +128). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12091,17 +12091,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox +1.5</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.6161</v>
+        <v>0.3669</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-160</v>
+        <v>173</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-153</v>
+        <v>162</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 61.6% (fair -160). Your call.</t>
+          <t>Model 36.7% (fair +173). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -12157,17 +12157,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Athletics -1.5</t>
+          <t>Athletics +1.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3839</v>
+        <v>0.6331</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>160</v>
+        <v>-173</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -12191,7 +12191,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 38.4% (fair +160). Your call.</t>
+          <t>Model 63.3% (fair -173). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -12227,13 +12227,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4317</v>
+        <v>0.4326</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -12257,7 +12257,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 43.2% (fair +132). Your call.</t>
+          <t>Model 43.3% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -12293,13 +12293,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.5683</v>
+        <v>0.5674</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-132</v>
+        <v>-131</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-138</v>
+        <v>-135</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -12323,7 +12323,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -132). Your call.</t>
+          <t>Model 56.7% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -12359,13 +12359,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5326</v>
+        <v>0.5533</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-114</v>
+        <v>-124</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-111</v>
+        <v>-113</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -12389,7 +12389,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12425,13 +12425,13 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4674</v>
+        <v>0.4467</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -12455,7 +12455,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12491,13 +12491,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.3875</v>
+        <v>0.3906</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -12521,7 +12521,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 38.8% (fair +158). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -12557,13 +12557,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.6125</v>
+        <v>0.6093999999999999</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-158</v>
+        <v>-156</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-160</v>
+        <v>-156</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -12587,7 +12587,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 61.3% (fair -158). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -12623,10 +12623,10 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.523841</v>
+        <v>0.53142</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-110</v>
+        <v>-113</v>
       </c>
       <c r="H35" s="15" t="n">
         <v>105</v>
@@ -12653,7 +12653,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -12689,10 +12689,10 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4761589999999999</v>
+        <v>0.46858</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="H36" s="15" t="n">
         <v>178</v>
@@ -12719,7 +12719,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -12755,7 +12755,7 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4436</v>
+        <v>0.4443</v>
       </c>
       <c r="G37" s="14" t="n">
         <v>125</v>
@@ -12821,7 +12821,7 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5564</v>
+        <v>0.5557000000000001</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>-125</v>
@@ -12887,13 +12887,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.5118</v>
+        <v>0.509</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -12917,7 +12917,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12953,10 +12953,10 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4882</v>
+        <v>0.491</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H40" s="15" t="n">
         <v>-108</v>
@@ -12983,7 +12983,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -13019,13 +13019,13 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.421</v>
+        <v>0.4209000000000001</v>
       </c>
       <c r="G41" s="14" t="n">
         <v>138</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -13085,7 +13085,7 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.579</v>
+        <v>0.5790999999999999</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>-138</v>
@@ -13147,17 +13147,17 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.3631</v>
+        <v>0.4617</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>175</v>
+        <v>117</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -13181,7 +13181,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 36.3% (fair +175). Your call.</t>
+          <t>Model 46.2% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -13213,17 +13213,17 @@
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.5531</v>
+        <v>0.5383</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>-124</v>
+        <v>-117</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -13247,7 +13247,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 53.8% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -13283,13 +13283,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.3935</v>
+        <v>0.3776</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -13313,7 +13313,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 39.4% (fair +154). Your call.</t>
+          <t>Model 37.8% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -13349,13 +13349,13 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.6065</v>
+        <v>0.6224000000000001</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-154</v>
+        <v>-165</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-153</v>
+        <v>162</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -13379,7 +13379,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 60.7% (fair -154). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -13415,7 +13415,7 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4812</v>
+        <v>0.4797</v>
       </c>
       <c r="G47" s="14" t="n">
         <v>108</v>
@@ -13445,7 +13445,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -13481,13 +13481,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5188</v>
+        <v>0.5203</v>
       </c>
       <c r="G48" s="14" t="n">
         <v>-108</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-104</v>
+        <v>-106</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -13511,7 +13511,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -13553,7 +13553,7 @@
         <v>-120</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -13943,13 +13943,13 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.511</v>
+        <v>0.5103</v>
       </c>
       <c r="G55" s="14" t="n">
         <v>-104</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>-102</v>
+        <v>-101</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -13973,7 +13973,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -104). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -14009,10 +14009,10 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4007</v>
+        <v>0.4014</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H56" s="15" t="n">
         <v>106</v>
@@ -14039,7 +14039,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +150). Your call.</t>
+          <t>Model 40.1% (fair +149). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14075,13 +14075,13 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4255</v>
+        <v>0.4218</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -14105,7 +14105,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14141,10 +14141,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5745</v>
+        <v>0.5782</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-135</v>
+        <v>-137</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>-156</v>
@@ -14171,7 +14171,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14207,7 +14207,7 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5219</v>
+        <v>0.5224</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>-109</v>
@@ -14273,7 +14273,7 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4781</v>
+        <v>0.4776</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>109</v>
@@ -14335,17 +14335,17 @@
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.5067</v>
+        <v>0.4885</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-103</v>
+        <v>105</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -14369,7 +14369,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4933</v>
+        <v>0.4191000000000001</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>103</v>
+        <v>139</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>-112</v>
+        <v>100</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14471,13 +14471,13 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.596</v>
+        <v>0.5914</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>-148</v>
+        <v>-145</v>
       </c>
       <c r="H63" s="15" t="n">
-        <v>-141</v>
+        <v>-138</v>
       </c>
       <c r="I63" s="13">
         <f>IF($H$63="","",IF($H$63&lt;0,-$H$63/(-$H$63+100),100/($H$63+100)))</f>
@@ -14501,7 +14501,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 59.6% (fair -148). Your call.</t>
+          <t>Model 59.1% (fair -145). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -14537,13 +14537,13 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.404</v>
+        <v>0.4086</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H64" s="15" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I64" s="13">
         <f>IF($H$64="","",IF($H$64&lt;0,-$H$64/(-$H$64+100),100/($H$64+100)))</f>
@@ -14567,7 +14567,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 40.4% (fair +148). Your call.</t>
+          <t>Model 40.9% (fair +145). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -14603,7 +14603,7 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4547</v>
+        <v>0.4539</v>
       </c>
       <c r="G65" s="14" t="n">
         <v>120</v>
@@ -14631,7 +14631,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -14667,7 +14667,7 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5453</v>
+        <v>0.5461</v>
       </c>
       <c r="G66" s="14" t="n">
         <v>-120</v>
@@ -14695,7 +14695,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -15371,10 +15371,10 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.5266</v>
+        <v>0.5278</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>-111</v>
+        <v>-112</v>
       </c>
       <c r="H77" s="15" t="n">
         <v>-117</v>
@@ -15401,7 +15401,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -111). Your call.</t>
+          <t>Model 52.8% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -15437,10 +15437,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.4734</v>
+        <v>0.4722</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>113</v>
@@ -15467,7 +15467,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 47.2% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -15767,13 +15767,13 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.5734</v>
+        <v>0.5699000000000001</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>-134</v>
+        <v>-133</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>-113</v>
+        <v>-108</v>
       </c>
       <c r="I83" s="13">
         <f>IF($H$83="","",IF($H$83&lt;0,-$H$83/(-$H$83+100),100/($H$83+100)))</f>
@@ -15797,7 +15797,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 57.3% (fair -134). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15833,10 +15833,10 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.4266</v>
+        <v>0.4301</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H84" s="15" t="n">
         <v>117</v>
@@ -15863,7 +15863,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 42.7% (fair +134). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -16295,10 +16295,10 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.4077</v>
+        <v>0.3587399999999999</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="H91" s="15" t="n">
         <v>133</v>
@@ -16325,7 +16325,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 40.8% (fair +145). Your call.</t>
+          <t>Model 35.9% (fair +179). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -16361,13 +16361,13 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.5923</v>
+        <v>0.6412600000000001</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>-145</v>
+        <v>-179</v>
       </c>
       <c r="H92" s="15" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="I92" s="13">
         <f>IF($H$92="","",IF($H$92&lt;0,-$H$92/(-$H$92+100),100/($H$92+100)))</f>
@@ -16391,7 +16391,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 64.1% (fair -179). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -16947,10 +16947,10 @@
         </is>
       </c>
       <c r="F101" s="13" t="n">
-        <v>0.4744</v>
+        <v>0.4728</v>
       </c>
       <c r="G101" s="14" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H101" s="15" t="n"/>
       <c r="I101" s="13">
@@ -16975,7 +16975,7 @@
       </c>
       <c r="N101" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 47.3% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O101" s="15" t="n"/>
@@ -17011,10 +17011,10 @@
         </is>
       </c>
       <c r="F102" s="13" t="n">
-        <v>0.5256</v>
+        <v>0.5272</v>
       </c>
       <c r="G102" s="14" t="n">
-        <v>-111</v>
+        <v>-112</v>
       </c>
       <c r="H102" s="15" t="n"/>
       <c r="I102" s="13">
@@ -17039,7 +17039,7 @@
       </c>
       <c r="N102" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 52.7% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O102" s="15" t="n"/>
@@ -17478,7 +17478,7 @@
         <v>204</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -17544,7 +17544,7 @@
         <v>-204</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-110</v>
+        <v>-120</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -17604,13 +17604,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4878</v>
+        <v>0.4951</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -17634,7 +17634,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -17670,13 +17670,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5122</v>
+        <v>0.5049</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-105</v>
+        <v>-102</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -17700,7 +17700,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -17732,17 +17732,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx -6.5</t>
+          <t>Minnesota Lynx -7.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4849254556076258</v>
+        <v>0.4536141029303052</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -17766,7 +17766,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -17798,17 +17798,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty +6.5</t>
+          <t>New York Liberty +7.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5150745443923742</v>
+        <v>0.5463858970696948</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-106</v>
+        <v>-120</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -17832,7 +17832,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -17874,7 +17874,7 @@
         <v>341</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>614</v>
+        <v>700</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -17940,7 +17940,7 @@
         <v>-341</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-115</v>
+        <v>-120</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -17996,17 +17996,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 173.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5622</v>
+        <v>0.5870644226482148</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-128</v>
+        <v>-142</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>117</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -18030,7 +18030,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -18062,17 +18062,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 173.5</t>
+          <t>Under 174.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4378</v>
+        <v>0.4129355773517852</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -18096,7 +18096,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 43.8% (fair +128). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -18128,17 +18128,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream -13.5</t>
+          <t>Atlanta Dream -14.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.442</v>
+        <v>0.4344</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 43.4% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -18194,17 +18194,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +13.5</t>
+          <t>Portland Fire +14.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5656</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-126</v>
+        <v>-130</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-103</v>
+        <v>105</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -18228,7 +18228,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 56.6% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -18392,17 +18392,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 170</t>
+          <t>Over 171</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.533</v>
+        <v>0.5556700048059063</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-114</v>
+        <v>-125</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -18426,7 +18426,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -18458,14 +18458,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 170</t>
+          <t>Under 171</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.444</v>
+        <v>0.4211299951940937</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>100</v>
@@ -18492,7 +18492,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 44.4% (fair +125). Your call.</t>
+          <t>Model 42.1% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -18524,17 +18524,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces -10.5</t>
+          <t>Las Vegas Aces -10</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4644</v>
+        <v>0.4626</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -18558,7 +18558,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +115). Your call.</t>
+          <t>Model 46.3% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -18590,17 +18590,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury +10.5</t>
+          <t>Phoenix Mercury +10</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5356000000000001</v>
+        <v>0.5063</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-115</v>
+        <v>-103</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -18624,7 +18624,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -18660,13 +18660,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.6204000000000001</v>
+        <v>0.6195999999999999</v>
       </c>
       <c r="G23" s="14" t="n">
         <v>-163</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-133</v>
+        <v>-138</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -18726,13 +18726,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.3796</v>
+        <v>0.3804</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>163</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -18792,10 +18792,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.3859</v>
+        <v>0.3875999999999999</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>156</v>
@@ -18822,7 +18822,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 38.6% (fair +159). Your call.</t>
+          <t>Model 38.8% (fair +158). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -18858,13 +18858,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.6141</v>
+        <v>0.6124000000000001</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-159</v>
+        <v>-158</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-194</v>
+        <v>-186</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -18888,7 +18888,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 61.4% (fair -159). Your call.</t>
+          <t>Model 61.2% (fair -158). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -18924,13 +18924,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.242</v>
+        <v>0.2307</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>313</v>
+        <v>333</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>270</v>
+        <v>317</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -18954,7 +18954,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 24.2% (fair +313). Your call.</t>
+          <t>Model 23.1% (fair +333). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -18990,10 +18990,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.758</v>
+        <v>0.7693</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-313</v>
+        <v>-333</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>-300</v>
@@ -19020,7 +19020,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 75.8% (fair -313). Your call.</t>
+          <t>Model 76.9% (fair -333). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -19056,13 +19056,13 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.3818</v>
+        <v>0.3901</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -19086,7 +19086,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 38.2% (fair +162). Your call.</t>
+          <t>Model 39.0% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -19122,13 +19122,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.6182</v>
+        <v>0.6099</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-162</v>
+        <v>-156</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-170</v>
+        <v>-163</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -19152,7 +19152,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 61.8% (fair -162). Your call.</t>
+          <t>Model 61.0% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-07-11 22:04Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-11.xlsx
+++ b/data/output/workbook/2026-07-11.xlsx
@@ -611,7 +611,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10267950"/>
+    <ext cx="10125075" cy="10648950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11 17:01</t>
+          <t>2026-07-11 18:03</t>
         </is>
       </c>
     </row>
@@ -6762,7 +6762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q79"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6779,903 +6779,903 @@
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="29" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
         <is>
           <t>Cleveland Guardians offense vs Miami Marlins defense</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="30" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B66" s="30" t="inlineStr">
+      <c r="B69" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C66" s="30" t="inlineStr">
+      <c r="C69" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D66" s="30" t="inlineStr">
+      <c r="D69" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E66" s="30" t="inlineStr">
+      <c r="E69" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F66" s="30" t="inlineStr">
+      <c r="F69" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G66" s="30" t="inlineStr">
+      <c r="G69" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H66" s="30" t="inlineStr">
+      <c r="H69" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I66" s="30" t="inlineStr">
+      <c r="I69" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J66" s="30" t="inlineStr">
+      <c r="J69" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K66" s="30" t="inlineStr">
+      <c r="K69" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L66" s="30" t="inlineStr">
+      <c r="L69" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M66" s="30" t="inlineStr">
+      <c r="M69" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N66" s="30" t="inlineStr">
+      <c r="N69" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O66" s="30" t="inlineStr">
+      <c r="O69" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P66" s="30" t="inlineStr">
+      <c r="P69" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q66" s="30" t="inlineStr">
+      <c r="Q69" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B67" s="32" t="n">
-        <v>3.918</v>
-      </c>
-      <c r="C67" s="32" t="n">
-        <v>3.667</v>
-      </c>
-      <c r="D67" s="32" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="E67" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="F67" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G67" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="H67" s="36" t="inlineStr">
-        <is>
-          <t>22nd</t>
-        </is>
-      </c>
-      <c r="I67" s="32" t="inlineStr"/>
-      <c r="J67" s="33" t="inlineStr">
-        <is>
-          <t>9th</t>
-        </is>
-      </c>
-      <c r="K67" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L67" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="M67" s="32" t="n">
-        <v>4.133</v>
-      </c>
-      <c r="N67" s="32" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="O67" s="32" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="P67" s="32" t="n">
-        <v>4.274</v>
-      </c>
-      <c r="Q67" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B68" s="32" t="n">
-        <v>7.735</v>
-      </c>
-      <c r="C68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H68" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I68" s="32" t="inlineStr"/>
-      <c r="J68" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O68" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P68" s="32" t="n">
-        <v>7.694</v>
-      </c>
-      <c r="Q68" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>0.959</v>
-      </c>
-      <c r="C69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr"/>
-      <c r="J69" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O69" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>1.082</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B70" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="C70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3.918</v>
+      </c>
+      <c r="C70" s="32" t="n">
+        <v>3.667</v>
+      </c>
+      <c r="D70" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G70" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="36" t="inlineStr">
+        <is>
+          <t>22nd</t>
         </is>
       </c>
       <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J70" s="33" t="inlineStr">
+        <is>
+          <t>9th</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L70" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="M70" s="32" t="n">
+        <v>4.133</v>
+      </c>
+      <c r="N70" s="32" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="O70" s="32" t="n">
+        <v>3.7</v>
       </c>
       <c r="P70" s="32" t="n">
-        <v>8.531000000000001</v>
+        <v>4.274</v>
       </c>
       <c r="Q70" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B71" s="32" t="n">
+        <v>7.735</v>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr"/>
+      <c r="J71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P71" s="32" t="n">
+        <v>7.694</v>
+      </c>
+      <c r="Q71" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="31" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="C72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr"/>
+      <c r="J72" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O72" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P72" s="32" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="Q72" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="n">
+        <v>8.531000000000001</v>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B71" s="32" t="n">
+      <c r="B74" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="C71" s="32" t="n">
+      <c r="C74" s="32" t="n">
         <v>0.267</v>
       </c>
-      <c r="D71" s="32" t="n">
+      <c r="D74" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="E71" s="32" t="n">
+      <c r="E74" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="F71" s="32" t="n">
+      <c r="F74" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="G71" s="32" t="n">
+      <c r="G74" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="H71" s="34" t="inlineStr">
+      <c r="H74" s="34" t="inlineStr">
         <is>
           <t>11th</t>
         </is>
       </c>
-      <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="33" t="inlineStr">
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="33" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="K71" s="32" t="n">
+      <c r="K74" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L71" s="32" t="n">
+      <c r="L74" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="M71" s="32" t="n">
+      <c r="M74" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="N71" s="32" t="n">
+      <c r="N74" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="O71" s="32" t="n">
+      <c r="O74" s="32" t="n">
         <v>0.333</v>
       </c>
-      <c r="P71" s="32" t="n">
+      <c r="P74" s="32" t="n">
         <v>0.585</v>
       </c>
-      <c r="Q71" s="35" t="inlineStr">
+      <c r="Q74" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="29" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
         <is>
           <t>Miami Marlins offense vs Cleveland Guardians defense</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="30" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B74" s="30" t="inlineStr">
+      <c r="B77" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C74" s="30" t="inlineStr">
+      <c r="C77" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D74" s="30" t="inlineStr">
+      <c r="D77" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E74" s="30" t="inlineStr">
+      <c r="E77" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F74" s="30" t="inlineStr">
+      <c r="F77" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G74" s="30" t="inlineStr">
+      <c r="G77" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H74" s="30" t="inlineStr">
+      <c r="H77" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I74" s="30" t="inlineStr">
+      <c r="I77" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J74" s="30" t="inlineStr">
+      <c r="J77" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K74" s="30" t="inlineStr">
+      <c r="K77" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L74" s="30" t="inlineStr">
+      <c r="L77" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M74" s="30" t="inlineStr">
+      <c r="M77" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N74" s="30" t="inlineStr">
+      <c r="N77" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O74" s="30" t="inlineStr">
+      <c r="O77" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P74" s="30" t="inlineStr">
+      <c r="P77" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q74" s="30" t="inlineStr">
+      <c r="Q77" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B75" s="32" t="n">
-        <v>4.69</v>
-      </c>
-      <c r="C75" s="32" t="n">
-        <v>5.467</v>
-      </c>
-      <c r="D75" s="32" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="E75" s="32" t="n">
-        <v>6.067</v>
-      </c>
-      <c r="F75" s="32" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G75" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="H75" s="33" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I75" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J75" s="34" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K75" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L75" s="32" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="M75" s="32" t="n">
-        <v>3.933</v>
-      </c>
-      <c r="N75" s="32" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="O75" s="32" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="P75" s="32" t="n">
-        <v>4.106</v>
-      </c>
-      <c r="Q75" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B76" s="32" t="n">
-        <v>8.286</v>
-      </c>
-      <c r="C76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H76" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I76" s="32" t="inlineStr"/>
-      <c r="J76" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O76" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P76" s="32" t="n">
-        <v>7.939</v>
-      </c>
-      <c r="Q76" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>0.918</v>
-      </c>
-      <c r="C77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O77" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P77" s="32" t="n">
-        <v>1.143</v>
-      </c>
-      <c r="Q77" s="35" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B78" s="32" t="n">
-        <v>7.816</v>
-      </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>4.69</v>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>5.467</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>6.067</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H78" s="33" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J78" s="34" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>3.933</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="O78" s="32" t="n">
+        <v>4.1</v>
       </c>
       <c r="P78" s="32" t="n">
-        <v>9.388</v>
+        <v>4.106</v>
       </c>
       <c r="Q78" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="n">
+        <v>8.286</v>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr"/>
+      <c r="J79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P79" s="32" t="n">
+        <v>7.939</v>
+      </c>
+      <c r="Q79" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="31" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="C80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="inlineStr"/>
+      <c r="J80" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O80" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P80" s="32" t="n">
+        <v>1.143</v>
+      </c>
+      <c r="Q80" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>7.816</v>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>9.388</v>
+      </c>
+      <c r="Q81" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B79" s="32" t="n">
+      <c r="B82" s="32" t="n">
         <v>0.585</v>
       </c>
-      <c r="C79" s="32" t="n">
+      <c r="C82" s="32" t="n">
         <v>0.5669999999999999</v>
       </c>
-      <c r="D79" s="32" t="n">
+      <c r="D82" s="32" t="n">
         <v>0.65</v>
       </c>
-      <c r="E79" s="32" t="n">
+      <c r="E82" s="32" t="n">
         <v>0.733</v>
       </c>
-      <c r="F79" s="32" t="n">
+      <c r="F82" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="32" t="n">
+      <c r="G82" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="H79" s="36" t="inlineStr">
+      <c r="H82" s="36" t="inlineStr">
         <is>
           <t>23rd</t>
         </is>
       </c>
-      <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="34" t="inlineStr">
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="34" t="inlineStr">
         <is>
           <t>13th</t>
         </is>
       </c>
-      <c r="K79" s="32" t="n">
+      <c r="K82" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="L79" s="32" t="n">
+      <c r="L82" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="M79" s="32" t="n">
+      <c r="M82" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="N79" s="32" t="n">
+      <c r="N82" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="O79" s="32" t="n">
+      <c r="O82" s="32" t="n">
         <v>0.433</v>
       </c>
-      <c r="P79" s="32" t="n">
+      <c r="P82" s="32" t="n">
         <v>0.366</v>
       </c>
-      <c r="Q79" s="35" t="inlineStr">
+      <c r="Q82" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8828,17 +8828,17 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Tampa Bay Rays</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -8848,17 +8848,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners +1.5</t>
+          <t>Athletics +1.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6698999999999999</v>
+        <v>0.6388</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-203</v>
+        <v>-177</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 67.0% (fair -203). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8899,12 +8899,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Seattle Mariners @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -8914,17 +8914,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers +1.5</t>
+          <t>Seattle Mariners +1.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6496</v>
+        <v>0.6698999999999999</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-185</v>
+        <v>-203</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8948,7 +8948,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 65.0% (fair -185). Your call.</t>
+          <t>Model 67.0% (fair -203). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8960,17 +8960,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Athletics @ Chicago White Sox</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8980,14 +8980,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Athletics +1.5</t>
+          <t>Milwaukee Brewers +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6427</v>
+        <v>0.6496</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-180</v>
+        <v>-185</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>178</v>
@@ -9014,7 +9014,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 64.3% (fair -180). Your call.</t>
+          <t>Model 65.0% (fair -185). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9050,10 +9050,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6351</v>
+        <v>0.6437999999999999</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-174</v>
+        <v>-181</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>170</v>
@@ -9080,7 +9080,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9224,7 +9224,7 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -9234,27 +9234,27 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5385</v>
+        <v>0.4466</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-117</v>
+        <v>124</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>133</v>
+        <v>178</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -117). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9295,7 +9295,7 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Seattle Mariners @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -9310,17 +9310,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Over 8</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5973000000000001</v>
+        <v>0.5554</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-148</v>
+        <v>-125</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 59.7% (fair -148). Your call.</t>
+          <t>Model 55.5% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9361,32 +9361,32 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates -1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4466</v>
+        <v>0.5434</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>124</v>
+        <v>-119</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>178</v>
+        <v>122</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9410,7 +9410,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9427,7 +9427,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Tampa Bay Rays</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
@@ -9442,17 +9442,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5554</v>
+        <v>0.5605</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-125</v>
+        <v>-128</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 56.0% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9493,12 +9493,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -9512,13 +9512,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5424</v>
+        <v>0.5354</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-119</v>
+        <v>-115</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9542,7 +9542,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -119). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -9574,11 +9574,11 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5354</v>
+        <v>0.5339</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>-115</v>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9644,10 +9644,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5555</v>
+        <v>0.5463</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-125</v>
+        <v>-120</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>109</v>
@@ -9674,7 +9674,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -9691,12 +9691,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -9706,17 +9706,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5339</v>
+        <v>0.518</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-115</v>
+        <v>-107</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9757,12 +9757,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>Phoenix Mercury @ Las Vegas Aces</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9772,17 +9772,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 169.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5172</v>
+        <v>0.5402</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-107</v>
+        <v>-117</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9823,12 +9823,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Las Vegas Aces</t>
+          <t>Portland Fire @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9838,17 +9838,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 169.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.539</v>
+        <v>0.5397999999999999</v>
       </c>
       <c r="G20" s="14" t="n">
         <v>-117</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9872,7 +9872,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9884,37 +9884,37 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Atlanta Dream</t>
+          <t>Atlanta Braves @ St. Louis Cardinals</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Over 174.5</t>
+          <t>St. Louis Cardinals -1.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5397999999999999</v>
+        <v>0.3991</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-117</v>
+        <v>151</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>104</v>
+        <v>174</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9938,7 +9938,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 39.9% (fair +151). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9950,37 +9950,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Athletics @ Chicago White Sox</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5473</v>
+        <v>0.648</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-121</v>
+        <v>-184</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>-147</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 64.8% (fair -184). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10016,17 +10016,17 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Philadelphia Phillies @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -10036,17 +10036,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5681</v>
+        <v>0.4784</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-132</v>
+        <v>109</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-108</v>
+        <v>127</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10070,7 +10070,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -132). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10087,32 +10087,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Braves @ St. Louis Cardinals</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals -1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.3991</v>
+        <v>0.5402</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>151</v>
+        <v>-117</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>174</v>
+        <v>100</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10136,7 +10136,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +151). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10153,32 +10153,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Detroit Tigers</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5256</v>
+        <v>0.4859</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-111</v>
+        <v>106</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10202,7 +10202,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10214,17 +10214,17 @@
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -10234,17 +10234,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.648</v>
+        <v>0.5716</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-184</v>
+        <v>-133</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-147</v>
+        <v>-113</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10268,7 +10268,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 64.8% (fair -184). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10280,37 +10280,37 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Detroit Tigers</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>22:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Chicago Cubs -1.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4779</v>
+        <v>0.4607</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10351,32 +10351,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Philadelphia Phillies @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4859</v>
+        <v>0.5158</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>106</v>
+        <v>-107</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10400,7 +10400,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 48.6% (fair +106). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10412,37 +10412,37 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs -1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.4607</v>
+        <v>0.482</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -10466,7 +10466,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 48.2% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -11567,7 +11567,7 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4828</v>
+        <v>0.482</v>
       </c>
       <c r="G19" s="14" t="n">
         <v>107</v>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 48.2% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -11633,7 +11633,7 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5172</v>
+        <v>0.518</v>
       </c>
       <c r="G20" s="14" t="n">
         <v>-107</v>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 51.8% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11699,7 +11699,7 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4625</v>
+        <v>0.4633</v>
       </c>
       <c r="G21" s="14" t="n">
         <v>116</v>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 46.3% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11765,7 +11765,7 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5375</v>
+        <v>0.5367</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>-116</v>
@@ -11795,7 +11795,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 53.7% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -11831,10 +11831,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4518915</v>
+        <v>0.453894</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>117</v>
@@ -11861,7 +11861,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 45.4% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11897,10 +11897,10 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5481085</v>
+        <v>0.546106</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-121</v>
+        <v>-120</v>
       </c>
       <c r="H24" s="15" t="n">
         <v>133</v>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11963,10 +11963,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5555</v>
+        <v>0.5463</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-125</v>
+        <v>-120</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>109</v>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 54.6% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12029,10 +12029,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.3538</v>
+        <v>0.3626</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>108</v>
@@ -12059,7 +12059,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 35.4% (fair +183). Your call.</t>
+          <t>Model 36.3% (fair +176). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12095,10 +12095,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.3649</v>
+        <v>0.3562</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>165</v>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 36.5% (fair +174). Your call.</t>
+          <t>Model 35.6% (fair +181). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -12161,10 +12161,10 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.6351</v>
+        <v>0.6437999999999999</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-174</v>
+        <v>-181</v>
       </c>
       <c r="H28" s="15" t="n">
         <v>170</v>
@@ -12191,7 +12191,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -12755,7 +12755,7 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4576</v>
+        <v>0.4566</v>
       </c>
       <c r="G37" s="14" t="n">
         <v>119</v>
@@ -12785,7 +12785,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +119). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12821,7 +12821,7 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5424</v>
+        <v>0.5434</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>-119</v>
@@ -12851,7 +12851,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -119). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12887,10 +12887,10 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.502</v>
+        <v>0.5011</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-101</v>
+        <v>-100</v>
       </c>
       <c r="H39" s="15" t="n">
         <v>111</v>
@@ -12917,7 +12917,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12953,10 +12953,10 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.498</v>
+        <v>0.4989</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H40" s="15" t="n">
         <v>-112</v>
@@ -12983,7 +12983,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -13943,10 +13943,10 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.5973000000000001</v>
+        <v>0.5605</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>-148</v>
+        <v>-128</v>
       </c>
       <c r="H55" s="15" t="n">
         <v>109</v>
@@ -13973,7 +13973,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 59.7% (fair -148). Your call.</t>
+          <t>Model 56.0% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -14009,10 +14009,10 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.3141999999999999</v>
+        <v>0.3489</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>218</v>
+        <v>187</v>
       </c>
       <c r="H56" s="15" t="n">
         <v>104</v>
@@ -14039,7 +14039,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 31.4% (fair +218). Your call.</t>
+          <t>Model 34.9% (fair +187). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14075,10 +14075,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.439</v>
+        <v>0.4368</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>144</v>
@@ -14105,7 +14105,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 43.9% (fair +128). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14141,10 +14141,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5609999999999999</v>
+        <v>0.5631999999999999</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-128</v>
+        <v>-129</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>-150</v>
@@ -14171,7 +14171,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14207,7 +14207,7 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5221</v>
+        <v>0.5216000000000001</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>-109</v>
@@ -14273,7 +14273,7 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4779</v>
+        <v>0.4784</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>109</v>
@@ -14339,13 +14339,13 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.4855</v>
+        <v>0.4593</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -14369,7 +14369,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14405,10 +14405,10 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.4221</v>
+        <v>0.4485</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="H62" s="15" t="n">
         <v>113</v>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14471,10 +14471,10 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.5935</v>
+        <v>0.5944</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>-146</v>
+        <v>-147</v>
       </c>
       <c r="H63" s="15" t="n">
         <v>-135</v>
@@ -14501,7 +14501,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 59.4% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -14537,10 +14537,10 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.4065</v>
+        <v>0.4056</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H64" s="15" t="n">
         <v>133</v>
@@ -14567,7 +14567,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 40.6% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -14603,10 +14603,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4434</v>
+        <v>0.4452</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -14631,7 +14631,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 44.3% (fair +126). Your call.</t>
+          <t>Model 44.5% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -14667,10 +14667,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5566</v>
+        <v>0.5548</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-126</v>
+        <v>-125</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -14695,7 +14695,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 55.7% (fair -126). Your call.</t>
+          <t>Model 55.5% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -15115,7 +15115,7 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.4858</v>
+        <v>0.4857</v>
       </c>
       <c r="G73" s="14" t="n">
         <v>106</v>
@@ -15179,7 +15179,7 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.5142</v>
+        <v>0.5143</v>
       </c>
       <c r="G74" s="14" t="n">
         <v>-106</v>
@@ -15243,10 +15243,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.3785</v>
+        <v>0.3603</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="H75" s="15" t="n"/>
       <c r="I75" s="13">
@@ -15271,7 +15271,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 37.9% (fair +164). Your call.</t>
+          <t>Model 36.0% (fair +178). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -15307,10 +15307,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.6215000000000001</v>
+        <v>0.6397</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-164</v>
+        <v>-178</v>
       </c>
       <c r="H76" s="15" t="n"/>
       <c r="I76" s="13">
@@ -15335,7 +15335,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 62.2% (fair -164). Your call.</t>
+          <t>Model 64.0% (fair -178). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -15371,13 +15371,13 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.5177</v>
+        <v>0.5233</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>-107</v>
+        <v>-110</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>-113</v>
+        <v>-122</v>
       </c>
       <c r="I77" s="13">
         <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
@@ -15401,7 +15401,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -107). Your call.</t>
+          <t>Model 52.3% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -15437,10 +15437,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.4823</v>
+        <v>0.4767</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>122</v>
@@ -15467,7 +15467,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +107). Your call.</t>
+          <t>Model 47.7% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="E79" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 7</t>
         </is>
       </c>
       <c r="F79" s="13" t="n">
@@ -15509,7 +15509,7 @@
         <v>-117</v>
       </c>
       <c r="H79" s="15" t="n">
-        <v>133</v>
+        <v>-104</v>
       </c>
       <c r="I79" s="13">
         <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
@@ -15565,17 +15565,17 @@
       </c>
       <c r="E80" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Under 7</t>
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.4615</v>
+        <v>0.3647</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>117</v>
+        <v>174</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -15599,7 +15599,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +117). Your call.</t>
+          <t>Model 36.5% (fair +174). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -16295,13 +16295,13 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.5681</v>
+        <v>0.5716</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>-132</v>
+        <v>-133</v>
       </c>
       <c r="H91" s="15" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="I91" s="13">
         <f>IF($H$91="","",IF($H$91&lt;0,-$H$91/(-$H$91+100),100/($H$91+100)))</f>
@@ -16325,7 +16325,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -132). Your call.</t>
+          <t>Model 57.2% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -16361,10 +16361,10 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.4319</v>
+        <v>0.4284</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H92" s="15" t="n">
         <v>117</v>
@@ -16391,7 +16391,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 43.2% (fair +132). Your call.</t>
+          <t>Model 42.8% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -16427,10 +16427,10 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.5228</v>
+        <v>0.5196</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="H93" s="15" t="n">
         <v>104</v>
@@ -16457,7 +16457,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 52.3% (fair -110). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -16493,13 +16493,13 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.4772</v>
+        <v>0.4804</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H94" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I94" s="13">
         <f>IF($H$94="","",IF($H$94&lt;0,-$H$94/(-$H$94+100),100/($H$94+100)))</f>
@@ -16523,7 +16523,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 47.7% (fair +110). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -17087,13 +17087,13 @@
         </is>
       </c>
       <c r="F103" s="13" t="n">
-        <v>0.4647</v>
+        <v>0.4654</v>
       </c>
       <c r="G103" s="14" t="n">
         <v>115</v>
       </c>
       <c r="H103" s="15" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="I103" s="13">
         <f>IF($H$103="","",IF($H$103&lt;0,-$H$103/(-$H$103+100),100/($H$103+100)))</f>
@@ -17153,7 +17153,7 @@
         </is>
       </c>
       <c r="F104" s="13" t="n">
-        <v>0.443</v>
+        <v>0.4423</v>
       </c>
       <c r="G104" s="14" t="n">
         <v>126</v>
@@ -17183,7 +17183,7 @@
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>Model 44.3% (fair +126). Your call.</t>
+          <t>Model 44.2% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O104" s="15" t="n"/>
@@ -17351,7 +17351,7 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.4837</v>
+        <v>0.4834000000000001</v>
       </c>
       <c r="G107" s="14" t="n">
         <v>107</v>
@@ -17381,7 +17381,7 @@
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O107" s="15" t="n"/>
@@ -17417,7 +17417,7 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.5163</v>
+        <v>0.5165999999999999</v>
       </c>
       <c r="G108" s="14" t="n">
         <v>-107</v>
@@ -17447,7 +17447,7 @@
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O108" s="15" t="n"/>
@@ -17483,10 +17483,10 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>0.5256</v>
+        <v>0.5158</v>
       </c>
       <c r="G109" s="14" t="n">
-        <v>-111</v>
+        <v>-107</v>
       </c>
       <c r="H109" s="15" t="n">
         <v>108</v>
@@ -17513,7 +17513,7 @@
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O109" s="15" t="n"/>
@@ -17549,10 +17549,10 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.4744</v>
+        <v>0.4842</v>
       </c>
       <c r="G110" s="14" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H110" s="15" t="n">
         <v>-104</v>
@@ -17579,7 +17579,7 @@
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O110" s="15" t="n"/>
@@ -17615,10 +17615,10 @@
         </is>
       </c>
       <c r="F111" s="13" t="n">
-        <v>0.6369</v>
+        <v>0.6389</v>
       </c>
       <c r="G111" s="14" t="n">
-        <v>-175</v>
+        <v>-177</v>
       </c>
       <c r="H111" s="15" t="n">
         <v>-186</v>
@@ -17645,7 +17645,7 @@
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>Model 63.7% (fair -175). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O111" s="15" t="n"/>
@@ -17681,10 +17681,10 @@
         </is>
       </c>
       <c r="F112" s="13" t="n">
-        <v>0.3631</v>
+        <v>0.3611</v>
       </c>
       <c r="G112" s="14" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H112" s="15" t="n">
         <v>180</v>
@@ -17711,7 +17711,7 @@
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>Model 36.3% (fair +175). Your call.</t>
+          <t>Model 36.1% (fair +177). Your call.</t>
         </is>
       </c>
       <c r="O112" s="15" t="n"/>
@@ -17747,13 +17747,13 @@
         </is>
       </c>
       <c r="F113" s="13" t="n">
-        <v>0.4119</v>
+        <v>0.4155</v>
       </c>
       <c r="G113" s="14" t="n">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H113" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I113" s="13">
         <f>IF($H$113="","",IF($H$113&lt;0,-$H$113/(-$H$113+100),100/($H$113+100)))</f>
@@ -17777,7 +17777,7 @@
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +143). Your call.</t>
+          <t>Model 41.5% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O113" s="15" t="n"/>
@@ -17813,10 +17813,10 @@
         </is>
       </c>
       <c r="F114" s="13" t="n">
-        <v>0.5881</v>
+        <v>0.5845</v>
       </c>
       <c r="G114" s="14" t="n">
-        <v>-143</v>
+        <v>-141</v>
       </c>
       <c r="H114" s="15" t="n">
         <v>-127</v>
@@ -17843,7 +17843,7 @@
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -143). Your call.</t>
+          <t>Model 58.5% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O114" s="15" t="n"/>
@@ -17879,10 +17879,10 @@
         </is>
       </c>
       <c r="F115" s="13" t="n">
-        <v>0.4332</v>
+        <v>0.4219000000000001</v>
       </c>
       <c r="G115" s="14" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="H115" s="15" t="n">
         <v>127</v>
@@ -17909,7 +17909,7 @@
       </c>
       <c r="N115" s="19" t="inlineStr">
         <is>
-          <t>Model 43.3% (fair +131). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O115" s="15" t="n"/>
@@ -17945,10 +17945,10 @@
         </is>
       </c>
       <c r="F116" s="13" t="n">
-        <v>0.5668</v>
+        <v>0.5780999999999999</v>
       </c>
       <c r="G116" s="14" t="n">
-        <v>-131</v>
+        <v>-137</v>
       </c>
       <c r="H116" s="15" t="n">
         <v>-127</v>
@@ -17975,7 +17975,7 @@
       </c>
       <c r="N116" s="19" t="inlineStr">
         <is>
-          <t>Model 56.7% (fair -131). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O116" s="15" t="n"/>
@@ -18011,10 +18011,10 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.4745</v>
+        <v>0.4526</v>
       </c>
       <c r="G117" s="14" t="n">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="H117" s="15" t="n">
         <v>101</v>
@@ -18041,7 +18041,7 @@
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O117" s="15" t="n"/>
@@ -18077,10 +18077,10 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.4385000000000001</v>
+        <v>0.4605</v>
       </c>
       <c r="G118" s="14" t="n">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="H118" s="15" t="n">
         <v>105</v>
@@ -18107,7 +18107,7 @@
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>Model 43.9% (fair +128). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O118" s="15" t="n"/>
@@ -18143,10 +18143,10 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.3922</v>
+        <v>0.3958</v>
       </c>
       <c r="G119" s="14" t="n">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H119" s="15" t="n">
         <v>165</v>
@@ -18173,7 +18173,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 39.2% (fair +155). Your call.</t>
+          <t>Model 39.6% (fair +153). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -18209,10 +18209,10 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.6078</v>
+        <v>0.6042000000000001</v>
       </c>
       <c r="G120" s="14" t="n">
-        <v>-155</v>
+        <v>-153</v>
       </c>
       <c r="H120" s="15" t="n">
         <v>-165</v>
@@ -18239,7 +18239,7 @@
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 60.4% (fair -153). Your call.</t>
         </is>
       </c>
       <c r="O120" s="15" t="n"/>
@@ -18275,7 +18275,7 @@
         </is>
       </c>
       <c r="F121" s="13" t="n">
-        <v>0.4544484</v>
+        <v>0.4539864</v>
       </c>
       <c r="G121" s="14" t="n">
         <v>120</v>
@@ -18341,7 +18341,7 @@
         </is>
       </c>
       <c r="F122" s="13" t="n">
-        <v>0.5455516</v>
+        <v>0.5460136</v>
       </c>
       <c r="G122" s="14" t="n">
         <v>-120</v>
@@ -18407,10 +18407,10 @@
         </is>
       </c>
       <c r="F123" s="13" t="n">
-        <v>0.5473</v>
+        <v>0.5402</v>
       </c>
       <c r="G123" s="14" t="n">
-        <v>-121</v>
+        <v>-117</v>
       </c>
       <c r="H123" s="15" t="n">
         <v>100</v>
@@ -18437,7 +18437,7 @@
       </c>
       <c r="N123" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O123" s="15" t="n"/>
@@ -18473,10 +18473,10 @@
         </is>
       </c>
       <c r="F124" s="13" t="n">
-        <v>0.4527</v>
+        <v>0.4598</v>
       </c>
       <c r="G124" s="14" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H124" s="15" t="n">
         <v>104</v>
@@ -18503,7 +18503,7 @@
       </c>
       <c r="N124" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O124" s="15" t="n"/>
@@ -18539,10 +18539,10 @@
         </is>
       </c>
       <c r="F125" s="13" t="n">
-        <v>0.3573</v>
+        <v>0.3612</v>
       </c>
       <c r="G125" s="14" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H125" s="15" t="n">
         <v>160</v>
@@ -18569,7 +18569,7 @@
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>Model 35.7% (fair +180). Your call.</t>
+          <t>Model 36.1% (fair +177). Your call.</t>
         </is>
       </c>
       <c r="O125" s="15" t="n"/>
@@ -18605,13 +18605,13 @@
         </is>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.6427</v>
+        <v>0.6388</v>
       </c>
       <c r="G126" s="14" t="n">
-        <v>-180</v>
+        <v>-177</v>
       </c>
       <c r="H126" s="15" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="I126" s="13">
         <f>IF($H$126="","",IF($H$126&lt;0,-$H$126/(-$H$126+100),100/($H$126+100)))</f>
@@ -18635,7 +18635,7 @@
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>Model 64.3% (fair -180). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O126" s="15" t="n"/>
@@ -18799,13 +18799,13 @@
         </is>
       </c>
       <c r="F129" s="13" t="n">
-        <v>0.4944</v>
+        <v>0.4912</v>
       </c>
       <c r="G129" s="14" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H129" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I129" s="13">
         <f>IF($H$129="","",IF($H$129&lt;0,-$H$129/(-$H$129+100),100/($H$129+100)))</f>
@@ -18829,7 +18829,7 @@
       </c>
       <c r="N129" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O129" s="15" t="n"/>
@@ -18865,10 +18865,10 @@
         </is>
       </c>
       <c r="F130" s="13" t="n">
-        <v>0.5056</v>
+        <v>0.5087999999999999</v>
       </c>
       <c r="G130" s="14" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="H130" s="15" t="n">
         <v>-108</v>
@@ -18895,7 +18895,7 @@
       </c>
       <c r="N130" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O130" s="15" t="n"/>
@@ -19191,7 +19191,7 @@
         </is>
       </c>
       <c r="F135" s="13" t="n">
-        <v>0.4728</v>
+        <v>0.4711</v>
       </c>
       <c r="G135" s="14" t="n">
         <v>112</v>
@@ -19219,7 +19219,7 @@
       </c>
       <c r="N135" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +112). Your call.</t>
+          <t>Model 47.1% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O135" s="15" t="n"/>
@@ -19255,7 +19255,7 @@
         </is>
       </c>
       <c r="F136" s="13" t="n">
-        <v>0.5272</v>
+        <v>0.5289</v>
       </c>
       <c r="G136" s="14" t="n">
         <v>-112</v>
@@ -19283,7 +19283,7 @@
       </c>
       <c r="N136" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -112). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O136" s="15" t="n"/>
@@ -19319,10 +19319,10 @@
         </is>
       </c>
       <c r="F137" s="13" t="n">
-        <v>0.5175999999999999</v>
+        <v>0.5135999999999999</v>
       </c>
       <c r="G137" s="14" t="n">
-        <v>-107</v>
+        <v>-106</v>
       </c>
       <c r="H137" s="15" t="n">
         <v>100</v>
@@ -19349,7 +19349,7 @@
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -107). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O137" s="15" t="n"/>
@@ -19385,10 +19385,10 @@
         </is>
       </c>
       <c r="F138" s="13" t="n">
-        <v>0.4824000000000001</v>
+        <v>0.4864000000000001</v>
       </c>
       <c r="G138" s="14" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H138" s="15" t="n">
         <v>104</v>
@@ -19415,7 +19415,7 @@
       </c>
       <c r="N138" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +107). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O138" s="15" t="n"/>
@@ -19451,10 +19451,10 @@
         </is>
       </c>
       <c r="F139" s="13" t="n">
-        <v>0.3967</v>
+        <v>0.3959</v>
       </c>
       <c r="G139" s="14" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H139" s="15" t="n">
         <v>150</v>
@@ -19481,7 +19481,7 @@
       </c>
       <c r="N139" s="19" t="inlineStr">
         <is>
-          <t>Model 39.7% (fair +152). Your call.</t>
+          <t>Model 39.6% (fair +153). Your call.</t>
         </is>
       </c>
       <c r="O139" s="15" t="n"/>
@@ -19517,10 +19517,10 @@
         </is>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.6032999999999999</v>
+        <v>0.6041000000000001</v>
       </c>
       <c r="G140" s="14" t="n">
-        <v>-152</v>
+        <v>-153</v>
       </c>
       <c r="H140" s="15" t="n">
         <v>-145</v>
@@ -19547,7 +19547,7 @@
       </c>
       <c r="N140" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 60.4% (fair -153). Your call.</t>
         </is>
       </c>
       <c r="O140" s="15" t="n"/>
@@ -19711,10 +19711,10 @@
         </is>
       </c>
       <c r="F143" s="13" t="n">
-        <v>0.5327</v>
+        <v>0.5241</v>
       </c>
       <c r="G143" s="14" t="n">
-        <v>-114</v>
+        <v>-110</v>
       </c>
       <c r="H143" s="15" t="n"/>
       <c r="I143" s="13">
@@ -19739,7 +19739,7 @@
       </c>
       <c r="N143" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O143" s="15" t="n"/>
@@ -19775,10 +19775,10 @@
         </is>
       </c>
       <c r="F144" s="13" t="n">
-        <v>0.4673</v>
+        <v>0.4759</v>
       </c>
       <c r="G144" s="14" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H144" s="15" t="n"/>
       <c r="I144" s="13">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="N144" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O144" s="15" t="n"/>
@@ -19839,10 +19839,10 @@
         </is>
       </c>
       <c r="F145" s="13" t="n">
-        <v>0.4819</v>
+        <v>0.4881</v>
       </c>
       <c r="G145" s="14" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H145" s="15" t="n">
         <v>104</v>
@@ -19869,7 +19869,7 @@
       </c>
       <c r="N145" s="19" t="inlineStr">
         <is>
-          <t>Model 48.2% (fair +108). Your call.</t>
+          <t>Model 48.8% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O145" s="15" t="n"/>
@@ -19905,10 +19905,10 @@
         </is>
       </c>
       <c r="F146" s="13" t="n">
-        <v>0.5181</v>
+        <v>0.5119</v>
       </c>
       <c r="G146" s="14" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="H146" s="15" t="n">
         <v>100</v>
@@ -19935,7 +19935,7 @@
       </c>
       <c r="N146" s="19" t="inlineStr">
         <is>
-          <t>Model 51.8% (fair -108). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O146" s="15" t="n"/>
@@ -19971,7 +19971,7 @@
         </is>
       </c>
       <c r="F147" s="13" t="n">
-        <v>0.5966</v>
+        <v>0.5974</v>
       </c>
       <c r="G147" s="14" t="n">
         <v>-148</v>
@@ -20037,7 +20037,7 @@
         </is>
       </c>
       <c r="F148" s="13" t="n">
-        <v>0.4034</v>
+        <v>0.4026</v>
       </c>
       <c r="G148" s="14" t="n">
         <v>148</v>
@@ -20646,7 +20646,7 @@
         <v>312</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>275</v>
+        <v>310</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -20772,7 +20772,7 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.539</v>
+        <v>0.5402</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>-117</v>
@@ -20802,7 +20802,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -20838,13 +20838,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.461</v>
+        <v>0.4598</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>117</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -20868,7 +20868,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -20910,7 +20910,7 @@
         <v>116</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -20976,7 +20976,7 @@
         <v>-116</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -21036,10 +21036,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.6175</v>
+        <v>0.6054</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-161</v>
+        <v>-153</v>
       </c>
       <c r="H17" s="15" t="n"/>
       <c r="I17" s="13">
@@ -21064,7 +21064,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 61.8% (fair -161). Your call.</t>
+          <t>Model 60.5% (fair -153). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -21100,10 +21100,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.3825</v>
+        <v>0.3946</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="H18" s="15" t="n"/>
       <c r="I18" s="13">
@@ -21128,7 +21128,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 38.2% (fair +161). Your call.</t>
+          <t>Model 39.5% (fair +153). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -21627,22 +21627,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>0.2497</v>
+        <v>0.2495</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.409</v>
+        <v>0.4105</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>-55.98</v>
+        <v>-54.56</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>-10.96</v>
+        <v>-10.62</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>4.41</v>
@@ -21658,22 +21658,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>0.2502</v>
+        <v>0.2499</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.4062</v>
+        <v>0.4079</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>-54.78</v>
+        <v>-53.36</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>-12.09</v>
+        <v>-11.7</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>6.29</v>
@@ -21762,7 +21762,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=389, ECE 0.044 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=390, ECE 0.043 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -21895,16 +21895,16 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0.6404</v>
+        <v>0.6402</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.5682</v>
+        <v>0.5778</v>
       </c>
       <c r="E22" s="27" t="n">
-        <v>-0.0722</v>
+        <v>-0.0625</v>
       </c>
     </row>
     <row r="23">

</xml_diff>